<commit_message>
Ajustes nos textos do checklist
</commit_message>
<xml_diff>
--- a/checklists/estudo_caso_1/checklist_estudo_caso_1.xlsx
+++ b/checklists/estudo_caso_1/checklist_estudo_caso_1.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="40">
   <si>
     <t>Modelo</t>
   </si>
@@ -49,7 +49,7 @@
     <t>Identificação correta de afirmações</t>
   </si>
   <si>
-    <t>Nenhum claim indevido; seção corretamente vazia.</t>
+    <t>Nenhuma afirmação indevida; seção corretamente vazia.</t>
   </si>
   <si>
     <t>Contexto preservado</t>
@@ -91,46 +91,40 @@
     <t>Llama 8B</t>
   </si>
   <si>
-    <t>Não encontrou erros, mas também não inventou nenhum.</t>
-  </si>
-  <si>
-    <t>Sem erros listados; nada indevido citado.</t>
-  </si>
-  <si>
-    <t>Nenhuma identificação feita erroneamente.</t>
-  </si>
-  <si>
-    <t>Sugestões mantêm sentido, exceto pequena inconsistência.</t>
-  </si>
-  <si>
-    <t>Trecho longo identificado corretamente.</t>
+    <t>Não encontrou erros reais no texto, mas também não inventou nenhum.</t>
+  </si>
+  <si>
+    <t>Os erros reais não foram listados nem localizados, mas não houve nenhum apontamento indevido</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Trecho longo identificado corretamente, mas não identificou todos os erros de clareza</t>
   </si>
   <si>
     <t>Sugestões formais, porém uma sugestão fora do trecho analisado.</t>
   </si>
   <si>
-    <t>Segue formato esperado.</t>
-  </si>
-  <si>
     <t>Há leve inconsistência sobre 'Copilot', mas não é alucinação.</t>
   </si>
   <si>
     <t>Llama 70B</t>
   </si>
   <si>
-    <t>Erros citados realmente aparecem no texto.</t>
+    <t>Não detectou todos os erros reais do texto. Nem todos os diagnósticos e correções são adequados.</t>
   </si>
   <si>
     <t>Todos os trechos constam no documento.</t>
   </si>
   <si>
-    <t>As afirmações existem, porém as recomendações de citação foram exageradas.</t>
-  </si>
-  <si>
-    <t>Sugestões preservam o significado.</t>
-  </si>
-  <si>
-    <t>Períodos longos corretamente identificados.</t>
+    <t>As afirmações existem, porém as recomendações de citação foram desnecessárias.</t>
+  </si>
+  <si>
+    <t>Exige citações desnecessárias</t>
+  </si>
+  <si>
+    <t>Período longo corretamente identificado, mas os outros diagnósticos de clareza foram exagerados ou genéricos.</t>
   </si>
   <si>
     <t>Sugestões mantêm formalidade.</t>
@@ -143,7 +137,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -159,6 +153,11 @@
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -189,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -199,6 +198,15 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -420,7 +428,7 @@
     <col customWidth="1" min="1" max="1" width="15.43"/>
     <col customWidth="1" min="2" max="2" width="36.14"/>
     <col customWidth="1" min="3" max="3" width="32.57"/>
-    <col customWidth="1" min="4" max="4" width="68.0"/>
+    <col customWidth="1" min="4" max="4" width="67.57"/>
     <col customWidth="1" min="5" max="6" width="8.71"/>
   </cols>
   <sheetData>
@@ -476,7 +484,7 @@
       <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -532,7 +540,7 @@
       <c r="C8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -560,7 +568,7 @@
       <c r="C10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>26</v>
       </c>
     </row>
@@ -574,7 +582,7 @@
       <c r="C11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="4" t="s">
         <v>27</v>
       </c>
     </row>
@@ -589,7 +597,7 @@
         <v>11</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -602,8 +610,11 @@
       <c r="C13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>29</v>
+      <c r="D13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="14">
@@ -616,8 +627,8 @@
       <c r="C14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>30</v>
+      <c r="D14" s="4" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="15">
@@ -631,7 +642,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16">
@@ -644,8 +655,8 @@
       <c r="C16" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>32</v>
+      <c r="D16" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="17">
@@ -659,12 +670,12 @@
         <v>23</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>5</v>
@@ -672,13 +683,13 @@
       <c r="C18" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>35</v>
+      <c r="D18" s="4" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>5</v>
@@ -687,12 +698,12 @@
         <v>8</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>10</v>
@@ -700,13 +711,13 @@
       <c r="C20" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
+      <c r="D20" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21">
       <c r="A21" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>10</v>
@@ -714,13 +725,13 @@
       <c r="C21" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
+      <c r="D21" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22">
       <c r="A22" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>15</v>
@@ -728,13 +739,13 @@
       <c r="C22" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
+      <c r="D22" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23">
       <c r="A23" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>15</v>
@@ -743,12 +754,12 @@
         <v>18</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24">
       <c r="A24" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>20</v>
@@ -756,13 +767,13 @@
       <c r="C24" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
+    <row r="25">
       <c r="A25" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>20</v>
@@ -771,7 +782,7 @@
         <v>23</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1"/>

</xml_diff>